<commit_message>
Added {666,669} for Squads, Added {66,67} for FutSquads (2025-06-28 16:44:03 UTC)
</commit_message>
<xml_diff>
--- a/result/pc64/Squads/669/fifa_ng_db_1.db_Changelogs/TablesChangelog.xlsx
+++ b/result/pc64/Squads/669/fifa_ng_db_1.db_Changelogs/TablesChangelog.xlsx
@@ -14,7 +14,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Added'!$A$1:$A$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Removed'!$A$1:$A$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Modified'!$A$1:$A$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Modified'!$A$1:$A$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -60,12 +60,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -484,10 +481,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -497,113 +494,8 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>cmplayers</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>competition</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>competitionballs</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>dcplayernames</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>default_mentalities</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>default_teamsheets</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>fixtures</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>leagueteamlinks</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>playerformdiff</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>players</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>smplayers</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>teamformdiff</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>teamplayerlinks</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>teams</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>version</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:A16"/>
+  <autoFilter ref="A1:A1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>